<commit_message>
MP orders: long-short 10/19 changes executed at 10/19 close; Troy 10/20 queued
Long-short (10/19 close): FST -1, Unitest -1, Simmtech +1, L&C Bio +1, CS Bearing +1, Finemtech 2% new
(fill prices checked against Naver 10/19 close). Troy (10/20 close, runs 20:05): Solum 2% new, Pan Ocean exit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/downloads/kosdaq_long_short_index_history.xlsx
+++ b/docs/downloads/kosdaq_long_short_index_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,196 +473,192 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>에스피지</t>
+          <t>에프에스티</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>058610</t>
+          <t>036810</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>79100</v>
+        <v>28650</v>
       </c>
       <c r="F2" t="n">
-        <v>205.0482</v>
+        <v>345.7839</v>
       </c>
       <c r="G2" t="n">
-        <v>16219315.2</v>
-      </c>
-      <c r="H2" t="n">
-        <v>-15.22</v>
-      </c>
+        <v>9906708.4</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>086450</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>25250</v>
+        <v>11600</v>
       </c>
       <c r="F3" t="n">
-        <v>768.6917999999999</v>
+        <v>854.0266</v>
       </c>
       <c r="G3" t="n">
-        <v>19409469.1</v>
+        <v>9906708.4</v>
       </c>
       <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>에이엘티</t>
+          <t>심텍</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>172670</t>
+          <t>222800</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>12510</v>
+        <v>131000</v>
       </c>
       <c r="F4" t="n">
-        <v>1443.4887</v>
+        <v>75.6237</v>
       </c>
       <c r="G4" t="n">
-        <v>18058043.3</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-11.28</v>
-      </c>
+        <v>9906708.4</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>심텍</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>222800</t>
+          <t>290650</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>126500</v>
+        <v>67100</v>
       </c>
       <c r="F5" t="n">
-        <v>383.5863</v>
+        <v>147.641</v>
       </c>
       <c r="G5" t="n">
-        <v>48523672.7</v>
+        <v>9906708.4</v>
       </c>
       <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>씨에스베어링</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>297090</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2485</v>
+        <v>4830</v>
       </c>
       <c r="F6" t="n">
-        <v>42403.6617</v>
+        <v>2051.0783</v>
       </c>
       <c r="G6" t="n">
-        <v>105373099.3</v>
+        <v>9906708.4</v>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RF머트리얼즈</t>
+          <t>파인엠텍</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>327260</t>
+          <t>441270</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>45500</v>
+        <v>9430</v>
       </c>
       <c r="F7" t="n">
-        <v>213.2909</v>
+        <v>2101.1046</v>
       </c>
       <c r="G7" t="n">
-        <v>9704734.5</v>
+        <v>19813416.7</v>
       </c>
       <c r="H7" t="inlineStr"/>
     </row>
@@ -674,29 +670,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>코스텍시스</t>
+          <t>에스피지</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>355150</t>
+          <t>058610</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>17880</v>
+        <v>79100</v>
       </c>
       <c r="F8" t="n">
-        <v>1085.5408</v>
+        <v>205.0482</v>
       </c>
       <c r="G8" t="n">
-        <v>19409469.1</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
+        <v>16219315.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-15.22</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -706,31 +704,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>388790</t>
+          <t>086450</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4460</v>
+        <v>25250</v>
       </c>
       <c r="F9" t="n">
-        <v>3137.3165</v>
+        <v>768.6917999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>13992431.8</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-17.83</v>
-      </c>
+        <v>19409469.1</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -740,110 +736,110 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>에스엠씨지</t>
+          <t>에이엘티</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>460870</t>
+          <t>172670</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3345</v>
+        <v>12510</v>
       </c>
       <c r="F10" t="n">
-        <v>11605.0637</v>
+        <v>1443.4887</v>
       </c>
       <c r="G10" t="n">
-        <v>38818938.1</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
+        <v>18058043.3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-11.28</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>제우스</t>
+          <t>심텍</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>079370</t>
+          <t>222800</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>12120</v>
+        <v>126500</v>
       </c>
       <c r="F11" t="n">
-        <v>820.878</v>
+        <v>383.5863</v>
       </c>
       <c r="G11" t="n">
-        <v>9949041.199999999</v>
+        <v>48523672.7</v>
       </c>
       <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>248000</v>
+        <v>2485</v>
       </c>
       <c r="F12" t="n">
-        <v>81.12909999999999</v>
+        <v>42403.6617</v>
       </c>
       <c r="G12" t="n">
-        <v>20120019.7</v>
-      </c>
-      <c r="H12" t="n">
-        <v>-19.98</v>
-      </c>
+        <v>105373099.3</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>RF머트리얼즈</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>327260</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -852,150 +848,150 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>222500</v>
+        <v>45500</v>
       </c>
       <c r="F13" t="n">
-        <v>178.8592</v>
+        <v>213.2909</v>
       </c>
       <c r="G13" t="n">
-        <v>39796164.7</v>
+        <v>9704734.5</v>
       </c>
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>알멕</t>
+          <t>코스텍시스</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>354320</t>
+          <t>355150</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>54500</v>
+        <v>17880</v>
       </c>
       <c r="F14" t="n">
-        <v>504.0447</v>
+        <v>1085.5408</v>
       </c>
       <c r="G14" t="n">
-        <v>27470436.6</v>
-      </c>
-      <c r="H14" t="n">
-        <v>24.43</v>
-      </c>
+        <v>19409469.1</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>에프에스티</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>036810</t>
+          <t>388790</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>32350</v>
+        <v>4460</v>
       </c>
       <c r="F15" t="n">
-        <v>314.5779</v>
+        <v>3137.3165</v>
       </c>
       <c r="G15" t="n">
-        <v>10176595.1</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
+        <v>13992431.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-17.83</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>유니테스트</t>
+          <t>에스엠씨지</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>086390</t>
+          <t>460870</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>13650</v>
+        <v>3345</v>
       </c>
       <c r="F16" t="n">
-        <v>745.5381</v>
+        <v>11605.0637</v>
       </c>
       <c r="G16" t="n">
-        <v>10176595.1</v>
+        <v>38818938.1</v>
       </c>
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>코세스</t>
+          <t>제우스</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>089890</t>
+          <t>079370</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>31950</v>
+        <v>12120</v>
       </c>
       <c r="F17" t="n">
-        <v>318.5163</v>
+        <v>820.878</v>
       </c>
       <c r="G17" t="n">
-        <v>10176595.1</v>
+        <v>9949041.199999999</v>
       </c>
       <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1010,66 +1006,68 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>250500</v>
+        <v>248000</v>
       </c>
       <c r="F18" t="n">
-        <v>81.2503</v>
+        <v>81.12909999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>20353190.3</v>
-      </c>
-      <c r="H18" t="inlineStr"/>
+        <v>20120019.7</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-19.98</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>에이엘티</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>172670</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>14100</v>
+        <v>222500</v>
       </c>
       <c r="F19" t="n">
-        <v>1443.4887</v>
+        <v>178.8592</v>
       </c>
       <c r="G19" t="n">
-        <v>20353190.3</v>
+        <v>39796164.7</v>
       </c>
       <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>코미코</t>
+          <t>알멕</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>183300</t>
+          <t>354320</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1078,16 +1076,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>31300</v>
+        <v>54500</v>
       </c>
       <c r="F20" t="n">
-        <v>1954.4702</v>
+        <v>504.0447</v>
       </c>
       <c r="G20" t="n">
-        <v>61174916</v>
+        <v>27470436.6</v>
       </c>
       <c r="H20" t="n">
-        <v>6.83</v>
+        <v>24.43</v>
       </c>
     </row>
     <row r="21">
@@ -1098,12 +1096,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>에프에스티</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>036810</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1112,13 +1110,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>2355</v>
+        <v>32350</v>
       </c>
       <c r="F21" t="n">
-        <v>65496.7248</v>
+        <v>314.5779</v>
       </c>
       <c r="G21" t="n">
-        <v>154244786.8</v>
+        <v>10176595.1</v>
       </c>
       <c r="H21" t="inlineStr"/>
     </row>
@@ -1130,27 +1128,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>네오셈</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>253590</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>15810</v>
+        <v>13650</v>
       </c>
       <c r="F22" t="n">
-        <v>5149.4473</v>
+        <v>745.5381</v>
       </c>
       <c r="G22" t="n">
-        <v>81412761.09999999</v>
+        <v>10176595.1</v>
       </c>
       <c r="H22" t="inlineStr"/>
     </row>
@@ -1162,12 +1160,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>코세스</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>290650</t>
+          <t>089890</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1176,10 +1174,10 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>56700</v>
+        <v>31950</v>
       </c>
       <c r="F23" t="n">
-        <v>179.4814</v>
+        <v>318.5163</v>
       </c>
       <c r="G23" t="n">
         <v>10176595.1</v>
@@ -1194,12 +1192,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>388790</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1208,10 +1206,10 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4660</v>
+        <v>250500</v>
       </c>
       <c r="F24" t="n">
-        <v>4367.6374</v>
+        <v>81.2503</v>
       </c>
       <c r="G24" t="n">
         <v>20353190.3</v>
@@ -1221,17 +1219,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HLB</t>
+          <t>에이엘티</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>028300</t>
+          <t>172670</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1240,30 +1238,30 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>44600</v>
+        <v>14100</v>
       </c>
       <c r="F25" t="n">
-        <v>1359.3974</v>
+        <v>1443.4887</v>
       </c>
       <c r="G25" t="n">
-        <v>60629123.5</v>
+        <v>20353190.3</v>
       </c>
       <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>한스바이오메드</t>
+          <t>코미코</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>042520</t>
+          <t>183300</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1272,147 +1270,143 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20300</v>
+        <v>31300</v>
       </c>
       <c r="F26" t="n">
-        <v>1162.9429</v>
+        <v>1954.4702</v>
       </c>
       <c r="G26" t="n">
-        <v>23607739.9</v>
+        <v>61174916</v>
       </c>
       <c r="H26" t="n">
-        <v>7.9</v>
+        <v>6.83</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>제우스</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>079370</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>13160</v>
+        <v>2355</v>
       </c>
       <c r="F27" t="n">
-        <v>767.846</v>
+        <v>65496.7248</v>
       </c>
       <c r="G27" t="n">
-        <v>10104853.9</v>
+        <v>154244786.8</v>
       </c>
       <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>네오셈</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>083650</t>
+          <t>253590</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>49050</v>
+        <v>15810</v>
       </c>
       <c r="F28" t="n">
-        <v>357.1039</v>
+        <v>5149.4473</v>
       </c>
       <c r="G28" t="n">
-        <v>17515946</v>
-      </c>
-      <c r="H28" t="n">
-        <v>-16.44</v>
-      </c>
+        <v>81412761.09999999</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>씨젠</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>096530</t>
+          <t>290650</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>37100</v>
+        <v>56700</v>
       </c>
       <c r="F29" t="n">
-        <v>604.321</v>
+        <v>179.4814</v>
       </c>
       <c r="G29" t="n">
-        <v>22420310.5</v>
-      </c>
-      <c r="H29" t="n">
-        <v>15.04</v>
-      </c>
+        <v>10176595.1</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>두산테스나</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>131970</t>
+          <t>388790</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>123700</v>
+        <v>4660</v>
       </c>
       <c r="F30" t="n">
-        <v>490.1303</v>
+        <v>4367.6374</v>
       </c>
       <c r="G30" t="n">
-        <v>60629123.5</v>
+        <v>20353190.3</v>
       </c>
       <c r="H30" t="inlineStr"/>
     </row>
@@ -1424,12 +1418,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>서진시스템</t>
+          <t>HLB</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>178320</t>
+          <t>028300</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1438,13 +1432,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>41150</v>
+        <v>44600</v>
       </c>
       <c r="F31" t="n">
-        <v>491.1229</v>
+        <v>1359.3974</v>
       </c>
       <c r="G31" t="n">
-        <v>20209707.8</v>
+        <v>60629123.5</v>
       </c>
       <c r="H31" t="inlineStr"/>
     </row>
@@ -1456,29 +1450,31 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>코미코</t>
+          <t>한스바이오메드</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>183300</t>
+          <t>042520</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>31500</v>
+        <v>20300</v>
       </c>
       <c r="F32" t="n">
-        <v>320.789</v>
+        <v>1162.9429</v>
       </c>
       <c r="G32" t="n">
-        <v>10104853.9</v>
-      </c>
-      <c r="H32" t="inlineStr"/>
+        <v>23607739.9</v>
+      </c>
+      <c r="H32" t="n">
+        <v>7.9</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1488,27 +1484,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>제우스</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>079370</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>228500</v>
+        <v>13160</v>
       </c>
       <c r="F33" t="n">
-        <v>88.4451</v>
+        <v>767.846</v>
       </c>
       <c r="G33" t="n">
-        <v>20209707.8</v>
+        <v>10104853.9</v>
       </c>
       <c r="H33" t="inlineStr"/>
     </row>
@@ -1520,12 +1516,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>에스티팜</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>237690</t>
+          <t>083650</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1534,16 +1530,16 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>88500</v>
+        <v>49050</v>
       </c>
       <c r="F34" t="n">
-        <v>900.2261</v>
+        <v>357.1039</v>
       </c>
       <c r="G34" t="n">
-        <v>79670012.59999999</v>
+        <v>17515946</v>
       </c>
       <c r="H34" t="n">
-        <v>-3.84</v>
+        <v>-16.44</v>
       </c>
     </row>
     <row r="35">
@@ -1554,12 +1550,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>씨젠</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>240810</t>
+          <t>096530</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1568,16 +1564,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>130100</v>
+        <v>37100</v>
       </c>
       <c r="F35" t="n">
-        <v>314.8563</v>
+        <v>604.321</v>
       </c>
       <c r="G35" t="n">
-        <v>40962809.6</v>
+        <v>22420310.5</v>
       </c>
       <c r="H35" t="n">
-        <v>8.33</v>
+        <v>15.04</v>
       </c>
     </row>
     <row r="36">
@@ -1588,27 +1584,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>두산테스나</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>131970</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2325</v>
+        <v>123700</v>
       </c>
       <c r="F36" t="n">
-        <v>21730.8686</v>
+        <v>490.1303</v>
       </c>
       <c r="G36" t="n">
-        <v>50524269.6</v>
+        <v>60629123.5</v>
       </c>
       <c r="H36" t="inlineStr"/>
     </row>
@@ -1620,12 +1616,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>서진시스템</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>290650</t>
+          <t>178320</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1634,13 +1630,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>64700</v>
+        <v>41150</v>
       </c>
       <c r="F37" t="n">
-        <v>468.5404</v>
+        <v>491.1229</v>
       </c>
       <c r="G37" t="n">
-        <v>30314561.7</v>
+        <v>20209707.8</v>
       </c>
       <c r="H37" t="inlineStr"/>
     </row>
@@ -1652,44 +1648,44 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>씨에스베어링</t>
+          <t>코미코</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>297090</t>
+          <t>183300</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>4670</v>
+        <v>31500</v>
       </c>
       <c r="F38" t="n">
-        <v>6491.3408</v>
+        <v>320.789</v>
       </c>
       <c r="G38" t="n">
-        <v>30314561.7</v>
+        <v>10104853.9</v>
       </c>
       <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1698,160 +1694,162 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2120</v>
+        <v>228500</v>
       </c>
       <c r="F39" t="n">
-        <v>63879.7502</v>
+        <v>88.4451</v>
       </c>
       <c r="G39" t="n">
-        <v>135425070.4</v>
+        <v>20209707.8</v>
       </c>
       <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>에스티팜</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>237690</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>2120</v>
+        <v>88500</v>
       </c>
       <c r="F40" t="n">
-        <v>3453.9051</v>
+        <v>900.2261</v>
       </c>
       <c r="G40" t="n">
-        <v>7322278.8</v>
-      </c>
-      <c r="H40" t="inlineStr"/>
+        <v>79670012.59999999</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-3.84</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>086450</t>
+          <t>240810</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>22900</v>
+        <v>130100</v>
       </c>
       <c r="F41" t="n">
-        <v>1397.6406</v>
+        <v>314.8563</v>
       </c>
       <c r="G41" t="n">
-        <v>32005969</v>
-      </c>
-      <c r="H41" t="inlineStr"/>
+        <v>40962809.6</v>
+      </c>
+      <c r="H41" t="n">
+        <v>8.33</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>인텔리안테크</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>189300</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>73600</v>
+        <v>2325</v>
       </c>
       <c r="F42" t="n">
-        <v>299.9614</v>
+        <v>21730.8686</v>
       </c>
       <c r="G42" t="n">
-        <v>22077158.2</v>
-      </c>
-      <c r="H42" t="n">
-        <v>16.09</v>
-      </c>
+        <v>50524269.6</v>
+      </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>290650</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2215</v>
+        <v>64700</v>
       </c>
       <c r="F43" t="n">
-        <v>28224.978</v>
+        <v>468.5404</v>
       </c>
       <c r="G43" t="n">
-        <v>62518326.2</v>
+        <v>30314561.7</v>
       </c>
       <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>알멕</t>
+          <t>씨에스베어링</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>354320</t>
+          <t>297090</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1860,62 +1858,62 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>43800</v>
+        <v>4670</v>
       </c>
       <c r="F44" t="n">
-        <v>504.0447</v>
+        <v>6491.3408</v>
       </c>
       <c r="G44" t="n">
-        <v>22077158.2</v>
+        <v>30314561.7</v>
       </c>
       <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>코스텍시스</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>355150</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>23650</v>
+        <v>2120</v>
       </c>
       <c r="F45" t="n">
-        <v>451.106</v>
+        <v>63879.7502</v>
       </c>
       <c r="G45" t="n">
-        <v>10668656.3</v>
+        <v>135425070.4</v>
       </c>
       <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>388790</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1924,86 +1922,86 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>5730</v>
+        <v>2120</v>
       </c>
       <c r="F46" t="n">
-        <v>3723.7893</v>
+        <v>3453.9051</v>
       </c>
       <c r="G46" t="n">
-        <v>21337312.7</v>
+        <v>7322278.8</v>
       </c>
       <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>티씨머티리얼즈</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>125020</t>
+          <t>086450</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>6080</v>
+        <v>22900</v>
       </c>
       <c r="F47" t="n">
-        <v>3255.5051</v>
+        <v>1397.6406</v>
       </c>
       <c r="G47" t="n">
-        <v>19793471.1</v>
-      </c>
-      <c r="H47" t="n">
-        <v>-2.59</v>
-      </c>
+        <v>32005969</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>에스티팜</t>
+          <t>인텔리안테크</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>237690</t>
+          <t>189300</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>95200</v>
+        <v>73600</v>
       </c>
       <c r="F48" t="n">
-        <v>221.6088</v>
+        <v>299.9614</v>
       </c>
       <c r="G48" t="n">
-        <v>21097154.4</v>
-      </c>
-      <c r="H48" t="inlineStr"/>
+        <v>22077158.2</v>
+      </c>
+      <c r="H48" t="n">
+        <v>16.09</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2018,34 +2016,34 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2205</v>
+        <v>2215</v>
       </c>
       <c r="F49" t="n">
-        <v>52623.2877</v>
+        <v>28224.978</v>
       </c>
       <c r="G49" t="n">
-        <v>116034349.3</v>
+        <v>62518326.2</v>
       </c>
       <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>알멕</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>083650</t>
+          <t>354320</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2054,30 +2052,30 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>58700</v>
+        <v>43800</v>
       </c>
       <c r="F50" t="n">
-        <v>357.1039</v>
+        <v>504.0447</v>
       </c>
       <c r="G50" t="n">
-        <v>20961998.6</v>
+        <v>22077158.2</v>
       </c>
       <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>유니테스트</t>
+          <t>코스텍시스</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>086390</t>
+          <t>355150</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2086,30 +2084,30 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>13250</v>
+        <v>23650</v>
       </c>
       <c r="F51" t="n">
-        <v>791.0188000000001</v>
+        <v>451.106</v>
       </c>
       <c r="G51" t="n">
-        <v>10480999.3</v>
+        <v>10668656.3</v>
       </c>
       <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>388790</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2118,30 +2116,30 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>2360</v>
+        <v>5730</v>
       </c>
       <c r="F52" t="n">
-        <v>66616.5209</v>
+        <v>3723.7893</v>
       </c>
       <c r="G52" t="n">
-        <v>157214989.3</v>
+        <v>21337312.7</v>
       </c>
       <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>실리콘투</t>
+          <t>티씨머티리얼즈</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>257720</t>
+          <t>125020</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2150,32 +2148,32 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>38300</v>
+        <v>6080</v>
       </c>
       <c r="F53" t="n">
-        <v>500.7861</v>
+        <v>3255.5051</v>
       </c>
       <c r="G53" t="n">
-        <v>19180107.1</v>
+        <v>19793471.1</v>
       </c>
       <c r="H53" t="n">
-        <v>-11.87</v>
+        <v>-2.59</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>코스텍시스</t>
+          <t>에스티팜</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>355150</t>
+          <t>237690</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2184,182 +2182,182 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>21150</v>
+        <v>95200</v>
       </c>
       <c r="F54" t="n">
-        <v>495.5555</v>
+        <v>221.6088</v>
       </c>
       <c r="G54" t="n">
-        <v>10480999.3</v>
+        <v>21097154.4</v>
       </c>
       <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>범한퓨얼셀</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>382900</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>23650</v>
+        <v>2205</v>
       </c>
       <c r="F55" t="n">
-        <v>832.6201</v>
+        <v>52623.2877</v>
       </c>
       <c r="G55" t="n">
-        <v>19691465.3</v>
-      </c>
-      <c r="H55" t="n">
-        <v>1.28</v>
-      </c>
+        <v>116034349.3</v>
+      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>제우스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>079370</t>
+          <t>083650</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>12310</v>
+        <v>58700</v>
       </c>
       <c r="F56" t="n">
-        <v>2480.1654</v>
+        <v>357.1039</v>
       </c>
       <c r="G56" t="n">
-        <v>30530836.4</v>
+        <v>20961998.6</v>
       </c>
       <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>한중엔시에스</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>107640</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>40650</v>
+        <v>13250</v>
       </c>
       <c r="F57" t="n">
-        <v>751.0661</v>
+        <v>791.0188000000001</v>
       </c>
       <c r="G57" t="n">
-        <v>30530836.4</v>
+        <v>10480999.3</v>
       </c>
       <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>283500</v>
+        <v>2360</v>
       </c>
       <c r="F58" t="n">
-        <v>71.795</v>
+        <v>66616.5209</v>
       </c>
       <c r="G58" t="n">
-        <v>20353890.9</v>
+        <v>157214989.3</v>
       </c>
       <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>실리콘투</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>257720</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>2390</v>
+        <v>38300</v>
       </c>
       <c r="F59" t="n">
-        <v>42581.3618</v>
+        <v>500.7861</v>
       </c>
       <c r="G59" t="n">
-        <v>101769454.6</v>
-      </c>
-      <c r="H59" t="inlineStr"/>
+        <v>19180107.1</v>
+      </c>
+      <c r="H59" t="n">
+        <v>-11.87</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2374,132 +2372,132 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>20450</v>
+        <v>21150</v>
       </c>
       <c r="F60" t="n">
-        <v>995.3003</v>
+        <v>495.5555</v>
       </c>
       <c r="G60" t="n">
-        <v>20353890.9</v>
+        <v>10480999.3</v>
       </c>
       <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>에프에스티</t>
+          <t>범한퓨얼셀</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>036810</t>
+          <t>382900</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>30200</v>
+        <v>23650</v>
       </c>
       <c r="F61" t="n">
-        <v>359.55</v>
+        <v>832.6201</v>
       </c>
       <c r="G61" t="n">
-        <v>10858410.6</v>
-      </c>
-      <c r="H61" t="inlineStr"/>
+        <v>19691465.3</v>
+      </c>
+      <c r="H61" t="n">
+        <v>1.28</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>주성엔지니어링</t>
+          <t>제우스</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>036930</t>
+          <t>079370</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>208500</v>
+        <v>12310</v>
       </c>
       <c r="F62" t="n">
-        <v>338</v>
+        <v>2480.1654</v>
       </c>
       <c r="G62" t="n">
-        <v>70473000</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0.97</v>
-      </c>
+        <v>30530836.4</v>
+      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>한스바이오메드</t>
+          <t>한중엔시에스</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>042520</t>
+          <t>107640</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>17720</v>
+        <v>40650</v>
       </c>
       <c r="F63" t="n">
-        <v>94.9217</v>
+        <v>751.0661</v>
       </c>
       <c r="G63" t="n">
-        <v>1682012.5</v>
+        <v>30530836.4</v>
       </c>
       <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>에스피지</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>058610</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2508,77 +2506,77 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>100500</v>
+        <v>283500</v>
       </c>
       <c r="F64" t="n">
-        <v>8.9518</v>
+        <v>71.795</v>
       </c>
       <c r="G64" t="n">
-        <v>899652.6</v>
+        <v>20353890.9</v>
       </c>
       <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>제우스</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>079370</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>11410</v>
+        <v>2390</v>
       </c>
       <c r="F65" t="n">
-        <v>6321.2722</v>
+        <v>42581.3618</v>
       </c>
       <c r="G65" t="n">
-        <v>72125715.8</v>
+        <v>101769454.6</v>
       </c>
       <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>유니테스트</t>
+          <t>코스텍시스</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>086390</t>
+          <t>355150</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>12880</v>
+        <v>20450</v>
       </c>
       <c r="F66" t="n">
-        <v>713.2027</v>
+        <v>995.3003</v>
       </c>
       <c r="G66" t="n">
-        <v>9186050.6</v>
+        <v>20353890.9</v>
       </c>
       <c r="H66" t="inlineStr"/>
     </row>
@@ -2590,12 +2588,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>에프에스티</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>086450</t>
+          <t>036810</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2604,13 +2602,13 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>21200</v>
+        <v>30200</v>
       </c>
       <c r="F67" t="n">
-        <v>120.8659</v>
+        <v>359.55</v>
       </c>
       <c r="G67" t="n">
-        <v>2562357.9</v>
+        <v>10858410.6</v>
       </c>
       <c r="H67" t="inlineStr"/>
     </row>
@@ -2622,29 +2620,31 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>코세스</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>089890</t>
+          <t>036930</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>27700</v>
+        <v>208500</v>
       </c>
       <c r="F68" t="n">
-        <v>161.1835</v>
+        <v>338</v>
       </c>
       <c r="G68" t="n">
-        <v>4464784.2</v>
-      </c>
-      <c r="H68" t="inlineStr"/>
+        <v>70473000</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.97</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>상신이디피</t>
+          <t>한스바이오메드</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>091580</t>
+          <t>042520</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2668,13 +2668,13 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>21500</v>
+        <v>17720</v>
       </c>
       <c r="F69" t="n">
-        <v>129.2032</v>
+        <v>94.9217</v>
       </c>
       <c r="G69" t="n">
-        <v>2777868.4</v>
+        <v>1682012.5</v>
       </c>
       <c r="H69" t="inlineStr"/>
     </row>
@@ -2686,12 +2686,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>씨젠</t>
+          <t>에스피지</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>096530</t>
+          <t>058610</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2700,13 +2700,13 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>34100</v>
+        <v>100500</v>
       </c>
       <c r="F70" t="n">
-        <v>21.679</v>
+        <v>8.9518</v>
       </c>
       <c r="G70" t="n">
-        <v>739252.6</v>
+        <v>899652.6</v>
       </c>
       <c r="H70" t="inlineStr"/>
     </row>
@@ -2718,27 +2718,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>한중엔시에스</t>
+          <t>제우스</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>107640</t>
+          <t>079370</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>40850</v>
+        <v>11410</v>
       </c>
       <c r="F71" t="n">
-        <v>123.3915</v>
+        <v>6321.2722</v>
       </c>
       <c r="G71" t="n">
-        <v>5040542.1</v>
+        <v>72125715.8</v>
       </c>
       <c r="H71" t="inlineStr"/>
     </row>
@@ -2750,27 +2750,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>308000</v>
+        <v>12880</v>
       </c>
       <c r="F72" t="n">
-        <v>9.1744</v>
+        <v>713.2027</v>
       </c>
       <c r="G72" t="n">
-        <v>2825715.8</v>
+        <v>9186050.6</v>
       </c>
       <c r="H72" t="inlineStr"/>
     </row>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>티씨머티리얼즈</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>125020</t>
+          <t>086450</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>6330</v>
+        <v>21200</v>
       </c>
       <c r="F73" t="n">
-        <v>50.5051</v>
+        <v>120.8659</v>
       </c>
       <c r="G73" t="n">
-        <v>319697.4</v>
+        <v>2562357.9</v>
       </c>
       <c r="H73" t="inlineStr"/>
     </row>
@@ -2814,12 +2814,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>코미코</t>
+          <t>코세스</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>183300</t>
+          <t>089890</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2828,13 +2828,13 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>31700</v>
+        <v>27700</v>
       </c>
       <c r="F74" t="n">
-        <v>158.7408</v>
+        <v>161.1835</v>
       </c>
       <c r="G74" t="n">
-        <v>5032084.2</v>
+        <v>4464784.2</v>
       </c>
       <c r="H74" t="inlineStr"/>
     </row>
@@ -2846,27 +2846,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>인텔리안테크</t>
+          <t>상신이디피</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>189300</t>
+          <t>091580</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>68700</v>
+        <v>21500</v>
       </c>
       <c r="F75" t="n">
-        <v>16.0386</v>
+        <v>129.2032</v>
       </c>
       <c r="G75" t="n">
-        <v>1101852.6</v>
+        <v>2777868.4</v>
       </c>
       <c r="H75" t="inlineStr"/>
     </row>
@@ -2878,27 +2878,27 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>씨젠</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>096530</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>256000</v>
+        <v>34100</v>
       </c>
       <c r="F76" t="n">
-        <v>45.4873</v>
+        <v>21.679</v>
       </c>
       <c r="G76" t="n">
-        <v>11644736.8</v>
+        <v>739252.6</v>
       </c>
       <c r="H76" t="inlineStr"/>
     </row>
@@ -2910,12 +2910,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>에스티팜</t>
+          <t>한중엔시에스</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>237690</t>
+          <t>107640</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2924,13 +2924,13 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>91100</v>
+        <v>40850</v>
       </c>
       <c r="F77" t="n">
-        <v>19.6174</v>
+        <v>123.3915</v>
       </c>
       <c r="G77" t="n">
-        <v>1787142.1</v>
+        <v>5040542.1</v>
       </c>
       <c r="H77" t="inlineStr"/>
     </row>
@@ -2942,27 +2942,27 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>240810</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>130900</v>
+        <v>308000</v>
       </c>
       <c r="F78" t="n">
-        <v>89.1437</v>
+        <v>9.1744</v>
       </c>
       <c r="G78" t="n">
-        <v>11668905.3</v>
+        <v>2825715.8</v>
       </c>
       <c r="H78" t="inlineStr"/>
     </row>
@@ -2974,27 +2974,27 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>티씨머티리얼즈</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>125020</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>2400</v>
+        <v>6330</v>
       </c>
       <c r="F79" t="n">
-        <v>32820.1843</v>
+        <v>50.5051</v>
       </c>
       <c r="G79" t="n">
-        <v>78768442.40000001</v>
+        <v>319697.4</v>
       </c>
       <c r="H79" t="inlineStr"/>
     </row>
@@ -3006,27 +3006,27 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>실리콘투</t>
+          <t>코미코</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>257720</t>
+          <t>183300</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>41150</v>
+        <v>31700</v>
       </c>
       <c r="F80" t="n">
-        <v>38.7861</v>
+        <v>158.7408</v>
       </c>
       <c r="G80" t="n">
-        <v>1596047.4</v>
+        <v>5032084.2</v>
       </c>
       <c r="H80" t="inlineStr"/>
     </row>
@@ -3038,12 +3038,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>RF머트리얼즈</t>
+          <t>인텔리안테크</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>327260</t>
+          <t>189300</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3052,13 +3052,13 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>49450</v>
+        <v>68700</v>
       </c>
       <c r="F81" t="n">
-        <v>83.90349999999999</v>
+        <v>16.0386</v>
       </c>
       <c r="G81" t="n">
-        <v>4149029</v>
+        <v>1101852.6</v>
       </c>
       <c r="H81" t="inlineStr"/>
     </row>
@@ -3070,27 +3070,27 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>범한퓨얼셀</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>382900</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>24750</v>
+        <v>256000</v>
       </c>
       <c r="F82" t="n">
-        <v>23.3799</v>
+        <v>45.4873</v>
       </c>
       <c r="G82" t="n">
-        <v>578652.6</v>
+        <v>11644736.8</v>
       </c>
       <c r="H82" t="inlineStr"/>
     </row>
@@ -3102,110 +3102,108 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>에스티팜</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>388790</t>
+          <t>237690</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>5450</v>
+        <v>91100</v>
       </c>
       <c r="F83" t="n">
-        <v>220.6267</v>
+        <v>19.6174</v>
       </c>
       <c r="G83" t="n">
-        <v>1202415.4</v>
+        <v>1787142.1</v>
       </c>
       <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>파마리서치</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>214450</t>
+          <t>240810</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>327000</v>
+        <v>130900</v>
       </c>
       <c r="F84" t="n">
-        <v>54</v>
+        <v>89.1437</v>
       </c>
       <c r="G84" t="n">
-        <v>17658000</v>
-      </c>
-      <c r="H84" t="n">
-        <v>-10.66</v>
-      </c>
+        <v>11668905.3</v>
+      </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>라이콤</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>388790</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>5130</v>
+        <v>2400</v>
       </c>
       <c r="F85" t="n">
-        <v>4001.7913</v>
+        <v>32820.1843</v>
       </c>
       <c r="G85" t="n">
-        <v>20529189.5</v>
+        <v>78768442.40000001</v>
       </c>
       <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>에프에스티</t>
+          <t>실리콘투</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>036810</t>
+          <t>257720</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3214,324 +3212,322 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>27100</v>
+        <v>41150</v>
       </c>
       <c r="F86" t="n">
-        <v>376</v>
+        <v>38.7861</v>
       </c>
       <c r="G86" t="n">
-        <v>10189600</v>
+        <v>1596047.4</v>
       </c>
       <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>리노공업</t>
+          <t>RF머트리얼즈</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>058470</t>
+          <t>327260</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>67600</v>
+        <v>49450</v>
       </c>
       <c r="F87" t="n">
-        <v>998</v>
+        <v>83.90349999999999</v>
       </c>
       <c r="G87" t="n">
-        <v>67464800</v>
-      </c>
-      <c r="H87" t="n">
-        <v>-3.57</v>
-      </c>
+        <v>4149029</v>
+      </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>유니테스트</t>
+          <t>범한퓨얼셀</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>086390</t>
+          <t>382900</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>11900</v>
+        <v>24750</v>
       </c>
       <c r="F88" t="n">
-        <v>856</v>
+        <v>23.3799</v>
       </c>
       <c r="G88" t="n">
-        <v>10186400</v>
+        <v>578652.6</v>
       </c>
       <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>코미코</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>183300</t>
+          <t>388790</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>29300</v>
+        <v>5450</v>
       </c>
       <c r="F89" t="n">
-        <v>2434</v>
+        <v>220.6267</v>
       </c>
       <c r="G89" t="n">
-        <v>71316200</v>
+        <v>1202415.4</v>
       </c>
       <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>파마리서치</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>240810</t>
+          <t>214450</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>119300</v>
+        <v>327000</v>
       </c>
       <c r="F90" t="n">
-        <v>171</v>
+        <v>54</v>
       </c>
       <c r="G90" t="n">
-        <v>20400300</v>
-      </c>
-      <c r="H90" t="inlineStr"/>
+        <v>17658000</v>
+      </c>
+      <c r="H90" t="n">
+        <v>-10.66</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>라이콤</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>388790</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>2445</v>
+        <v>5130</v>
       </c>
       <c r="F91" t="n">
-        <v>82456</v>
+        <v>4001.7913</v>
       </c>
       <c r="G91" t="n">
-        <v>201604920</v>
+        <v>20529189.5</v>
       </c>
       <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>한스바이오메드</t>
+          <t>에프에스티</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>042520</t>
+          <t>036810</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>18910</v>
+        <v>27100</v>
       </c>
       <c r="F92" t="n">
-        <v>1068.0212</v>
+        <v>376</v>
       </c>
       <c r="G92" t="n">
-        <v>20196280</v>
+        <v>10189600</v>
       </c>
       <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>씨젠</t>
+          <t>리노공업</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>096530</t>
+          <t>058470</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>32250</v>
+        <v>67600</v>
       </c>
       <c r="F93" t="n">
-        <v>626</v>
+        <v>998</v>
       </c>
       <c r="G93" t="n">
-        <v>20188500</v>
-      </c>
-      <c r="H93" t="inlineStr"/>
+        <v>67464800</v>
+      </c>
+      <c r="H93" t="n">
+        <v>-3.57</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>82500</v>
+        <v>11900</v>
       </c>
       <c r="F94" t="n">
-        <v>204</v>
+        <v>856</v>
       </c>
       <c r="G94" t="n">
-        <v>16830000</v>
-      </c>
-      <c r="H94" t="n">
-        <v>-8.640000000000001</v>
-      </c>
+        <v>10186400</v>
+      </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>코미코</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>183300</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>56800</v>
+        <v>29300</v>
       </c>
       <c r="F95" t="n">
-        <v>258</v>
+        <v>2434</v>
       </c>
       <c r="G95" t="n">
-        <v>14654400</v>
-      </c>
-      <c r="H95" t="n">
-        <v>-17.68</v>
-      </c>
+        <v>71316200</v>
+      </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>240810</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3540,271 +3536,273 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>83700</v>
+        <v>119300</v>
       </c>
       <c r="F96" t="n">
-        <v>120</v>
+        <v>171</v>
       </c>
       <c r="G96" t="n">
-        <v>10044000</v>
+        <v>20400300</v>
       </c>
       <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>실리콘투</t>
+          <t>KODEX 코스닥150선물인버스</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>257720</t>
+          <t>251340</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>43650</v>
+        <v>2445</v>
       </c>
       <c r="F97" t="n">
-        <v>462</v>
+        <v>82456</v>
       </c>
       <c r="G97" t="n">
-        <v>20166300</v>
+        <v>201604920</v>
       </c>
       <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>한스바이오메드</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>042520</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>59700</v>
+        <v>18910</v>
       </c>
       <c r="F98" t="n">
-        <v>169</v>
+        <v>1068.0212</v>
       </c>
       <c r="G98" t="n">
-        <v>10089300</v>
+        <v>20196280</v>
       </c>
       <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>유니테스트</t>
+          <t>씨젠</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>086390</t>
+          <t>096530</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>10930</v>
+        <v>32250</v>
       </c>
       <c r="F99" t="n">
-        <v>1833</v>
+        <v>626</v>
       </c>
       <c r="G99" t="n">
-        <v>20034690</v>
+        <v>20188500</v>
       </c>
       <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>086450</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>19850</v>
+        <v>82500</v>
       </c>
       <c r="F100" t="n">
-        <v>505</v>
+        <v>204</v>
       </c>
       <c r="G100" t="n">
-        <v>10024250</v>
-      </c>
-      <c r="H100" t="inlineStr"/>
+        <v>16830000</v>
+      </c>
+      <c r="H100" t="n">
+        <v>-8.640000000000001</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>코세스</t>
+          <t>에이비엘바이오</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>089890</t>
+          <t>298380</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>비중 확대</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>26350</v>
+        <v>56800</v>
       </c>
       <c r="F101" t="n">
-        <v>380</v>
+        <v>258</v>
       </c>
       <c r="G101" t="n">
-        <v>10013000</v>
-      </c>
-      <c r="H101" t="inlineStr"/>
+        <v>14654400</v>
+      </c>
+      <c r="H101" t="n">
+        <v>-17.68</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>오이솔루션</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>138080</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>편출</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>23500</v>
+        <v>83700</v>
       </c>
       <c r="F102" t="n">
-        <v>833</v>
+        <v>120</v>
       </c>
       <c r="G102" t="n">
-        <v>19575500</v>
-      </c>
-      <c r="H102" t="n">
-        <v>-2.08</v>
-      </c>
+        <v>10044000</v>
+      </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>실리콘투</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>257720</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>편입</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>85200</v>
+        <v>43650</v>
       </c>
       <c r="F103" t="n">
-        <v>118</v>
+        <v>462</v>
       </c>
       <c r="G103" t="n">
-        <v>10053600</v>
+        <v>20166300</v>
       </c>
       <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>인텔리안테크</t>
+          <t>에이비엘바이오</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>189300</t>
+          <t>298380</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>63400</v>
+        <v>59700</v>
       </c>
       <c r="F104" t="n">
-        <v>316</v>
+        <v>169</v>
       </c>
       <c r="G104" t="n">
-        <v>20034400</v>
+        <v>10089300</v>
       </c>
       <c r="H104" t="inlineStr"/>
     </row>
@@ -3816,27 +3814,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>240810</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>110300</v>
+        <v>10930</v>
       </c>
       <c r="F105" t="n">
-        <v>91</v>
+        <v>1833</v>
       </c>
       <c r="G105" t="n">
-        <v>10037300</v>
+        <v>20034690</v>
       </c>
       <c r="H105" t="inlineStr"/>
     </row>
@@ -3848,140 +3846,142 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>086450</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>비중 축소</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>66100</v>
+        <v>19850</v>
       </c>
       <c r="F106" t="n">
-        <v>152</v>
+        <v>505</v>
       </c>
       <c r="G106" t="n">
-        <v>10047200</v>
+        <v>10024250</v>
       </c>
       <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>에프에스티</t>
+          <t>코세스</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>036810</t>
+          <t>089890</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 확대</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>25800</v>
+        <v>26350</v>
       </c>
       <c r="F107" t="n">
-        <v>2713</v>
+        <v>380</v>
       </c>
       <c r="G107" t="n">
-        <v>69995400</v>
+        <v>10013000</v>
       </c>
       <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>주성엔지니어링</t>
+          <t>오이솔루션</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>036930</t>
+          <t>138080</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>편출</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>206500</v>
+        <v>23500</v>
       </c>
       <c r="F108" t="n">
-        <v>338</v>
+        <v>833</v>
       </c>
       <c r="G108" t="n">
-        <v>69797000</v>
-      </c>
-      <c r="H108" t="inlineStr"/>
+        <v>19575500</v>
+      </c>
+      <c r="H108" t="n">
+        <v>-2.08</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>리노공업</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>058470</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>70100</v>
+        <v>85200</v>
       </c>
       <c r="F109" t="n">
-        <v>998</v>
+        <v>118</v>
       </c>
       <c r="G109" t="n">
-        <v>69959800</v>
+        <v>10053600</v>
       </c>
       <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>에스피지</t>
+          <t>인텔리안테크</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>058610</t>
+          <t>189300</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3990,77 +3990,77 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>93300</v>
+        <v>63400</v>
       </c>
       <c r="F110" t="n">
-        <v>214</v>
+        <v>316</v>
       </c>
       <c r="G110" t="n">
-        <v>19966200</v>
+        <v>20034400</v>
       </c>
       <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>유니테스트</t>
+          <t>원익IPS</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>086390</t>
+          <t>240810</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>11300</v>
+        <v>110300</v>
       </c>
       <c r="F111" t="n">
-        <v>4424</v>
+        <v>91</v>
       </c>
       <c r="G111" t="n">
-        <v>49991200</v>
+        <v>10037300</v>
       </c>
       <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>에이비엘바이오</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>086450</t>
+          <t>298380</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>편입</t>
+          <t>비중 축소</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>19740</v>
+        <v>66100</v>
       </c>
       <c r="F112" t="n">
-        <v>2532</v>
+        <v>152</v>
       </c>
       <c r="G112" t="n">
-        <v>49981680</v>
+        <v>10047200</v>
       </c>
       <c r="H112" t="inlineStr"/>
     </row>
@@ -4072,12 +4072,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>코세스</t>
+          <t>에프에스티</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>089890</t>
+          <t>036810</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -4086,13 +4086,13 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>25150</v>
+        <v>25800</v>
       </c>
       <c r="F113" t="n">
-        <v>2385</v>
+        <v>2713</v>
       </c>
       <c r="G113" t="n">
-        <v>59982750</v>
+        <v>69995400</v>
       </c>
       <c r="H113" t="inlineStr"/>
     </row>
@@ -4104,12 +4104,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>상신이디피</t>
+          <t>주성엔지니어링</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>091580</t>
+          <t>036930</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4118,13 +4118,13 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>22050</v>
+        <v>206500</v>
       </c>
       <c r="F114" t="n">
-        <v>2267</v>
+        <v>338</v>
       </c>
       <c r="G114" t="n">
-        <v>49987350</v>
+        <v>69797000</v>
       </c>
       <c r="H114" t="inlineStr"/>
     </row>
@@ -4136,12 +4136,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>한중엔시에스</t>
+          <t>리노공업</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>107640</t>
+          <t>058470</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4150,13 +4150,13 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>43150</v>
+        <v>70100</v>
       </c>
       <c r="F115" t="n">
-        <v>1390</v>
+        <v>998</v>
       </c>
       <c r="G115" t="n">
-        <v>59978500</v>
+        <v>69959800</v>
       </c>
       <c r="H115" t="inlineStr"/>
     </row>
@@ -4168,12 +4168,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>에스피지</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>058610</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4182,13 +4182,13 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>310000</v>
+        <v>93300</v>
       </c>
       <c r="F116" t="n">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="G116" t="n">
-        <v>69750000</v>
+        <v>19966200</v>
       </c>
       <c r="H116" t="inlineStr"/>
     </row>
@@ -4200,12 +4200,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>티씨머티리얼즈</t>
+          <t>유니테스트</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>125020</t>
+          <t>086390</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -4214,13 +4214,13 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>6240</v>
+        <v>11300</v>
       </c>
       <c r="F117" t="n">
-        <v>3205</v>
+        <v>4424</v>
       </c>
       <c r="G117" t="n">
-        <v>19999200</v>
+        <v>49991200</v>
       </c>
       <c r="H117" t="inlineStr"/>
     </row>
@@ -4232,12 +4232,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>오이솔루션</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>138080</t>
+          <t>086450</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -4246,13 +4246,13 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>24000</v>
+        <v>19740</v>
       </c>
       <c r="F118" t="n">
-        <v>833</v>
+        <v>2532</v>
       </c>
       <c r="G118" t="n">
-        <v>19992000</v>
+        <v>49981680</v>
       </c>
       <c r="H118" t="inlineStr"/>
     </row>
@@ -4264,12 +4264,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>코세스</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>089890</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -4278,13 +4278,13 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>90300</v>
+        <v>25150</v>
       </c>
       <c r="F119" t="n">
-        <v>442</v>
+        <v>2385</v>
       </c>
       <c r="G119" t="n">
-        <v>39912600</v>
+        <v>59982750</v>
       </c>
       <c r="H119" t="inlineStr"/>
     </row>
@@ -4296,12 +4296,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>상신이디피</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>091580</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>279500</v>
+        <v>22050</v>
       </c>
       <c r="F120" t="n">
-        <v>357</v>
+        <v>2267</v>
       </c>
       <c r="G120" t="n">
-        <v>99781500</v>
+        <v>49987350</v>
       </c>
       <c r="H120" t="inlineStr"/>
     </row>
@@ -4328,12 +4328,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>파마리서치</t>
+          <t>한중엔시에스</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>214450</t>
+          <t>107640</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -4342,13 +4342,13 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>366000</v>
+        <v>43150</v>
       </c>
       <c r="F121" t="n">
-        <v>54</v>
+        <v>1390</v>
       </c>
       <c r="G121" t="n">
-        <v>19764000</v>
+        <v>59978500</v>
       </c>
       <c r="H121" t="inlineStr"/>
     </row>
@@ -4360,12 +4360,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>에스티팜</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>237690</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -4374,13 +4374,13 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>91000</v>
+        <v>310000</v>
       </c>
       <c r="F122" t="n">
-        <v>659</v>
+        <v>225</v>
       </c>
       <c r="G122" t="n">
-        <v>59969000</v>
+        <v>69750000</v>
       </c>
       <c r="H122" t="inlineStr"/>
     </row>
@@ -4392,12 +4392,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>원익IPS</t>
+          <t>티씨머티리얼즈</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>240810</t>
+          <t>125020</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -4406,13 +4406,13 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>120100</v>
+        <v>6240</v>
       </c>
       <c r="F123" t="n">
-        <v>666</v>
+        <v>3205</v>
       </c>
       <c r="G123" t="n">
-        <v>79986600</v>
+        <v>19999200</v>
       </c>
       <c r="H123" t="inlineStr"/>
     </row>
@@ -4424,12 +4424,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>KODEX 코스닥150선물인버스</t>
+          <t>오이솔루션</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>251340</t>
+          <t>138080</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4438,13 +4438,13 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>2405</v>
+        <v>24000</v>
       </c>
       <c r="F124" t="n">
-        <v>415800</v>
+        <v>833</v>
       </c>
       <c r="G124" t="n">
-        <v>999999000</v>
+        <v>19992000</v>
       </c>
       <c r="H124" t="inlineStr"/>
     </row>
@@ -4456,12 +4456,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4470,13 +4470,13 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>69000</v>
+        <v>90300</v>
       </c>
       <c r="F125" t="n">
-        <v>579</v>
+        <v>442</v>
       </c>
       <c r="G125" t="n">
-        <v>39951000</v>
+        <v>39912600</v>
       </c>
       <c r="H125" t="inlineStr"/>
     </row>
@@ -4488,12 +4488,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>RF머트리얼즈</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>327260</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -4502,13 +4502,13 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>42300</v>
+        <v>279500</v>
       </c>
       <c r="F126" t="n">
-        <v>709</v>
+        <v>357</v>
       </c>
       <c r="G126" t="n">
-        <v>29990700</v>
+        <v>99781500</v>
       </c>
       <c r="H126" t="inlineStr"/>
     </row>
@@ -4520,29 +4520,221 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
+          <t>파마리서치</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>214450</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>편입</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>366000</v>
+      </c>
+      <c r="F127" t="n">
+        <v>54</v>
+      </c>
+      <c r="G127" t="n">
+        <v>19764000</v>
+      </c>
+      <c r="H127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>에스티팜</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>237690</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>편입</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>91000</v>
+      </c>
+      <c r="F128" t="n">
+        <v>659</v>
+      </c>
+      <c r="G128" t="n">
+        <v>59969000</v>
+      </c>
+      <c r="H128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>원익IPS</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>240810</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>편입</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>120100</v>
+      </c>
+      <c r="F129" t="n">
+        <v>666</v>
+      </c>
+      <c r="G129" t="n">
+        <v>79986600</v>
+      </c>
+      <c r="H129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>KODEX 코스닥150선물인버스</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>251340</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>편입</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>2405</v>
+      </c>
+      <c r="F130" t="n">
+        <v>415800</v>
+      </c>
+      <c r="G130" t="n">
+        <v>999999000</v>
+      </c>
+      <c r="H130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>에이비엘바이오</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>298380</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>편입</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>69000</v>
+      </c>
+      <c r="F131" t="n">
+        <v>579</v>
+      </c>
+      <c r="G131" t="n">
+        <v>39951000</v>
+      </c>
+      <c r="H131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>RF머트리얼즈</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>327260</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>편입</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>42300</v>
+      </c>
+      <c r="F132" t="n">
+        <v>709</v>
+      </c>
+      <c r="G132" t="n">
+        <v>29990700</v>
+      </c>
+      <c r="H132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
           <t>범한퓨얼셀</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C133" t="inlineStr">
         <is>
           <t>382900</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D133" t="inlineStr">
         <is>
           <t>편입</t>
         </is>
       </c>
-      <c r="E127" t="n">
+      <c r="E133" t="n">
         <v>23350</v>
       </c>
-      <c r="F127" t="n">
+      <c r="F133" t="n">
         <v>856</v>
       </c>
-      <c r="G127" t="n">
+      <c r="G133" t="n">
         <v>19987600</v>
       </c>
-      <c r="H127" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>